<commit_message>
add links for ice skating, hockey, fitness class
</commit_message>
<xml_diff>
--- a/nsns_courses/2025课程列表.xlsx
+++ b/nsns_courses/2025课程列表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qiang\source\Repo\nsns_courses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2B49568-B493-4F48-9D56-DBAC0D9060D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E417D57-53E7-4302-943E-8E68FCA17E10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{2D772B29-792D-42CE-9C63-F3F9E4697AEC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{2D772B29-792D-42CE-9C63-F3F9E4697AEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sport Program" sheetId="5" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="148">
   <si>
     <t>龙舟课</t>
   </si>
@@ -454,9 +454,6 @@
     <t>https://docs.google.com/forms/d/e/1FAIpQLSe2R4VGrdyp5hbwsAl3cMKXGPG5CDtjxfxut47TyLQ8ee8dFQ/viewform</t>
   </si>
   <si>
-    <t>https://docs.google.com/forms/d/1FZcTQUhvcJojD4k9GwHexXaqTgfjvWzdiphtXJbEwGw/viewform</t>
-  </si>
-  <si>
     <t>https://docs.google.com/forms/d/12VdvC9_TAzsPVMRlHg8rCQ6bnxYCmuNkeejoMZKEnBM/viewform</t>
   </si>
   <si>
@@ -509,6 +506,12 @@
   </si>
   <si>
     <t>https://docs.google.com/forms/d/1VNnxFnUPsmZO9sAiZ9d3nONQ6Rza9zPG8NvCDJ66c-Q/viewform</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSdTtJLgaxA6-mn6JX1PGmyLDcM0BLHNusJ7KQcPGKhUuGzSZQ/viewform</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSeyGD7nJtJlcS-oTQu-WlXJ9yZ0W3M7qhuMepEGP6rh7SnXcw/viewform</t>
   </si>
 </sst>
 </file>
@@ -739,7 +742,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -767,10 +770,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="7" xfId="1" applyFill="1" applyBorder="1"/>
@@ -1501,10 +1503,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="D6" s="14" t="s">
         <v>130</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>131</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>38</v>
@@ -1671,7 +1673,7 @@
         <v>34</v>
       </c>
       <c r="G14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
@@ -1919,10 +1921,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -1933,7 +1935,7 @@
         <v>124</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1968,7 +1970,7 @@
         <v>117</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -2031,19 +2033,24 @@
       <c r="A18" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="18"/>
+      <c r="B18" s="16" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>59</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -2084,9 +2091,11 @@
     <hyperlink ref="B2" r:id="rId14" xr:uid="{A55D131C-1979-4B34-8810-4A382A8D3787}"/>
     <hyperlink ref="B6" r:id="rId15" xr:uid="{7B918585-13CD-4DF2-BB60-959CDA284858}"/>
     <hyperlink ref="B5" r:id="rId16" xr:uid="{9E390795-809C-4217-A61B-8957A0FF5B09}"/>
+    <hyperlink ref="B20" r:id="rId17" xr:uid="{E403B793-807C-4569-8BA1-9872B67F7FCB}"/>
+    <hyperlink ref="B18" r:id="rId18" xr:uid="{8D45A3FB-994F-4714-9D85-A792A7C192B8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId17"/>
+  <pageSetup orientation="portrait" r:id="rId19"/>
 </worksheet>
 </file>
 
@@ -2383,87 +2392,87 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="20" t="s">
-        <v>137</v>
-      </c>
-      <c r="B2" s="24" t="s">
         <v>136</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B3" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="B3" s="22" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B4" s="22" t="s">
         <v>139</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="24" t="s">
-        <v>141</v>
+      <c r="B5" s="23" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="23" t="s">
-        <v>142</v>
+      <c r="B6" s="22" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="26" t="s">
-        <v>143</v>
+      <c r="B7" s="25" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="24" t="s">
-        <v>144</v>
+      <c r="B8" s="23" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="23" t="s">
-        <v>145</v>
+      <c r="B9" s="22" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="24" t="s">
-        <v>146</v>
+      <c r="B10" s="23" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="23"/>
+      <c r="B11" s="22"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="24" t="s">
         <v>78</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update skiing class link
</commit_message>
<xml_diff>
--- a/nsns_courses/2025课程列表.xlsx
+++ b/nsns_courses/2025课程列表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qiang\source\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qiang\source\Repo\nsns_courses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FAF0B1F-421D-4A20-ABF4-07DD33684ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F379E903-728F-4070-B7AD-A093E24FCF98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25320" yWindow="270" windowWidth="25440" windowHeight="15270" xr2:uid="{2D772B29-792D-42CE-9C63-F3F9E4697AEC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D772B29-792D-42CE-9C63-F3F9E4697AEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sport Program" sheetId="5" r:id="rId1"/>
@@ -414,7 +414,7 @@
     <t>https://docs.google.com/forms/d/1GpNUO_OJbmDc943RwX3Vpj18Yg8G9H1crSmgxfTadY4/viewform</t>
   </si>
   <si>
-    <t>https://docs.google.com/forms/d/1V_1vHKX9TQL8-KQGWn9lwo7g_Ug-u7BK_nHp2rRCpK0/viewform</t>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSeGg0XQ-63OxklP8fGjwHyo5UiHlntxg2wemdVRWkHNx45eOA/viewform</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
add skii course link
</commit_message>
<xml_diff>
--- a/nsns_courses/2025课程列表.xlsx
+++ b/nsns_courses/2025课程列表.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qiang\source\Repo\nsns_courses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E417D57-53E7-4302-943E-8E68FCA17E10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F379E903-728F-4070-B7AD-A093E24FCF98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{2D772B29-792D-42CE-9C63-F3F9E4697AEC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D772B29-792D-42CE-9C63-F3F9E4697AEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sport Program" sheetId="5" r:id="rId1"/>
-    <sheet name="Sport Program English" sheetId="6" r:id="rId2"/>
-    <sheet name="Cognitive Program" sheetId="2" r:id="rId3"/>
-    <sheet name="Cognitive Program English" sheetId="7" r:id="rId4"/>
-    <sheet name="Summer Camp " sheetId="4" r:id="rId5"/>
+    <sheet name="Cognitive Skills Program" sheetId="2" r:id="rId2"/>
+    <sheet name="Creative Arts Program" sheetId="3" r:id="rId3"/>
+    <sheet name="Summer Camp " sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="116">
   <si>
     <t>龙舟课</t>
   </si>
@@ -175,6 +174,9 @@
   </si>
   <si>
     <t>一对一私课（16节课）Token支付</t>
+  </si>
+  <si>
+    <t>一对一私课（20节课）其他支付</t>
   </si>
   <si>
     <r>
@@ -346,6 +348,9 @@
     <t>https://docs.google.com/forms/d/198luAUmUyLfaq6JPTgbIovaYUgqacQnfdElrWIgx0Hk/viewform</t>
   </si>
   <si>
+    <t>https://docs.google.com/forms/d/1fH5105wBzPqZjBJrUNfTPmcdHongj2l8gL_FdEjYTmg/viewform</t>
+  </si>
+  <si>
     <t>https://docs.google.com/forms/d/14tQfrW-aPs8rLP6PVJhs5zB9LnP1IUQbF7xHfh6XD84/viewform</t>
   </si>
   <si>
@@ -409,109 +414,7 @@
     <t>https://docs.google.com/forms/d/1GpNUO_OJbmDc943RwX3Vpj18Yg8G9H1crSmgxfTadY4/viewform</t>
   </si>
   <si>
-    <t>https://docs.google.com/forms/d/1V_1vHKX9TQL8-KQGWn9lwo7g_Ug-u7BK_nHp2rRCpK0/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/12kbzpmJ5GLfdR5lioQuGtYTZKXr59bR6oCMDMBufkHU/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1r7po6lq-9aQGgoneS8MuGz9zOAMzSRdnKob_PZ_8ztk/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1bDn1U3WaNWEdYm0u8btWeWD17jc-zmP4WPFH6xRkmFU/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/e/1FAIpQLSemwhGB52x143_-ItvlVSeCNNlmwKQEy9en58ZJ_tez4t-CYQ/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1HqFPA9Vefm-Qlbgdsmvvi2LZ_to4KEZzMafMjnnENac/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1I7rr_ijzm6OI6EbIOQ0D8JnHxKSuq18DKrw6prbjpRE/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1HYoAKTkV3xxtQyaZdVYBC5rG3nKzE3A7oRn9ej_Koe0/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/17OUh6xPgldU7CHqBCbou0iV970QX3PMk1Uxt0WX-fcg/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1BGq6ivZJ6E1TU6Ljhj2VNHa_KEqibHPcr4NZgnSFxsc/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/e/1FAIpQLSfBv6Y5unweLEkyzeVm099yQUqMBdoKV0bHR5ddwW9vYWNpTA/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1NtDZONO_jXtod7a6QHikIh88-QS2t9yoynrqLe-P4EQ/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/13O8dnuyXSXX10Hln3Epg4XiHyi75CACGH5xW9_2QhQM/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1l1KNHRYHq_9RlkvnponG9ZIJIdzO3un_BackqKPfBJ4/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/e/1FAIpQLSe2R4VGrdyp5hbwsAl3cMKXGPG5CDtjxfxut47TyLQ8ee8dFQ/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/12VdvC9_TAzsPVMRlHg8rCQ6bnxYCmuNkeejoMZKEnBM/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1zZSVJ6lLLqsh7CjhQHXj_6-RHe1PAGtbIC67QaDgRMQ/viewform</t>
-  </si>
-  <si>
-    <t>私课</t>
-  </si>
-  <si>
-    <t>Paddleboard</t>
-  </si>
-  <si>
-    <t>URL? Location?</t>
-  </si>
-  <si>
-    <t>1 on 1 and group?</t>
-  </si>
-  <si>
-    <t>Richmond Hill， Whitchurch-Stouffville，Oakville，Markham</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1K_80pZpF4LkO0rET5xVbKIMQHpfWOCWyqWqiPzm0U68/viewform</t>
-  </si>
-  <si>
-    <t>机器人课1</t>
-  </si>
-  <si>
-    <t>机器人课2</t>
-  </si>
-  <si>
-    <t>机器人summer camp</t>
-  </si>
-  <si>
-    <t>https://www.cognitoforms.com/CodeNinjasRichmondHill/_2025SummerCampEnrollmentFormNSNS</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1TZsM71ch1cRuX62F5wQEhoO93PIvnURYQ-E_UOwJtso/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1i17KJuzeT62RBplNLfDk3pHXIqcKxtDzvxyKq9tISMI/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1Z4RagEQcaCsO9Ey1zOg2qJMMn-padRCE_Tbl0QDiZwo/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1zxW-jGQdQ1soeXj_NzWBEI2-kmNFf0DjZJzYL-KAhXA/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1G8g3OBqLMhTIjGCwo8bqiOMDYZOsywI64NTWu3bolU0/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/1VNnxFnUPsmZO9sAiZ9d3nONQ6Rza9zPG8NvCDJ66c-Q/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/e/1FAIpQLSdTtJLgaxA6-mn6JX1PGmyLDcM0BLHNusJ7KQcPGKhUuGzSZQ/viewform</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/forms/d/e/1FAIpQLSeyGD7nJtJlcS-oTQu-WlXJ9yZ0W3M7qhuMepEGP6rh7SnXcw/viewform</t>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSeGg0XQ-63OxklP8fGjwHyo5UiHlntxg2wemdVRWkHNx45eOA/viewform</t>
   </si>
 </sst>
 </file>
@@ -562,7 +465,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -593,50 +496,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor theme="4" tint="0.79998168889431442"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor theme="4" tint="0.59999389629810485"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor theme="4" tint="0.59999389629810485"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor theme="4" tint="0.79998168889431442"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="8">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -687,62 +548,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="0"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="0"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="0"/>
-      </right>
-      <top style="thin">
-        <color theme="0"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="0"/>
-      </right>
-      <top style="thin">
-        <color theme="0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0"/>
-      </left>
-      <right style="thin">
-        <color theme="0"/>
-      </right>
-      <top style="thin">
-        <color theme="0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -759,25 +570,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="7" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1015,8 +807,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1DE48A40-BBF7-4C2D-9CD8-461EBAD8184F}" name="Table5" displayName="Table5" ref="B1:G25" totalsRowShown="0" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5">
-  <autoFilter ref="B1:G25" xr:uid="{1DE48A40-BBF7-4C2D-9CD8-461EBAD8184F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1DE48A40-BBF7-4C2D-9CD8-461EBAD8184F}" name="Table5" displayName="Table5" ref="B1:G24" totalsRowShown="0" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5">
+  <autoFilter ref="B1:G24" xr:uid="{1DE48A40-BBF7-4C2D-9CD8-461EBAD8184F}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{7BA89182-689B-4A34-85EA-C4FEB4416A22}" name="报名链接"/>
     <tableColumn id="2" xr3:uid="{8A9D31D0-1A54-4F70-8C93-8D5784AD596E}" name="课程安排"/>
@@ -1030,8 +822,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3ECBEB19-8677-450F-A1C7-4C58E8D77A8F}" name="Table2" displayName="Table2" ref="A1:G12" totalsRowShown="0">
-  <autoFilter ref="A1:G12" xr:uid="{3ECBEB19-8677-450F-A1C7-4C58E8D77A8F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3ECBEB19-8677-450F-A1C7-4C58E8D77A8F}" name="Table2" displayName="Table2" ref="A1:G8" totalsRowShown="0">
+  <autoFilter ref="A1:G8" xr:uid="{3ECBEB19-8677-450F-A1C7-4C58E8D77A8F}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{BD9C8922-8FE0-4641-B057-B085C13AF57A}" name="课程"/>
     <tableColumn id="2" xr3:uid="{D0D1A6FB-D014-4920-95A5-C6263F3E649E}" name="报名链接" dataCellStyle="Hyperlink"/>
@@ -1046,6 +838,22 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{938F0ACB-D05A-40CC-A479-19379C0BA82C}" name="Table3" displayName="Table3" ref="A1:G6" totalsRowShown="0">
+  <autoFilter ref="A1:G6" xr:uid="{938F0ACB-D05A-40CC-A479-19379C0BA82C}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{B4B152D2-5A72-40FD-8B93-1B68F29CBAFD}" name="课程"/>
+    <tableColumn id="2" xr3:uid="{A3DCAB0A-79D3-42E3-A4AB-490E5D8A3023}" name="报名链接" dataCellStyle="Hyperlink"/>
+    <tableColumn id="7" xr3:uid="{B241A288-A554-462C-8336-7277E254A32C}" name="课程安排" dataCellStyle="Hyperlink"/>
+    <tableColumn id="3" xr3:uid="{23734466-121A-4CF5-9C7C-F2417452CB26}" name="上课形式"/>
+    <tableColumn id="4" xr3:uid="{4FAE7445-1951-4503-A878-ED75E145201E}" name="每课时长"/>
+    <tableColumn id="5" xr3:uid="{01B2F079-EEF2-424B-8619-85E466113E8F}" name="上课日期"/>
+    <tableColumn id="6" xr3:uid="{EF688D66-ABC5-4752-B8BA-46BD15CD36B1}" name="地点"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{46A561AF-64E5-49B2-939D-0053BD404BA3}" name="Table4" displayName="Table4" ref="A1:C6" totalsRowShown="0">
   <autoFilter ref="A1:C6" xr:uid="{46A561AF-64E5-49B2-939D-0053BD404BA3}"/>
   <tableColumns count="3">
@@ -1374,7 +1182,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75E5E6B0-1EB1-4F61-854E-1DF46E8E8B9E}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.77734375" customWidth="1"/>
@@ -1386,15 +1194,15 @@
     <col min="7" max="7" width="89.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D1" t="s">
         <v>24</v>
@@ -1409,15 +1217,15 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="17.399999999999999" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="17.399999999999999" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D2" t="s">
         <v>20</v>
@@ -1426,21 +1234,21 @@
         <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D3" t="s">
         <v>29</v>
@@ -1452,15 +1260,15 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D4" t="s">
         <v>40</v>
@@ -1469,21 +1277,21 @@
         <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
@@ -1492,179 +1300,178 @@
         <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="E6" s="14" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="14"/>
-      <c r="G6" s="15"/>
-      <c r="H6"/>
-      <c r="I6"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
-        <v>55</v>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>3</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C8" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" t="s">
-        <v>64</v>
+      <c r="F8" t="s">
+        <v>73</v>
       </c>
       <c r="G8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
-        <v>4</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C9" t="s">
         <v>61</v>
       </c>
       <c r="D9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" t="s">
         <v>20</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E10" t="s">
         <v>38</v>
       </c>
-      <c r="F9" t="s">
-        <v>72</v>
-      </c>
-      <c r="G9" t="s">
+      <c r="F10" t="s">
+        <v>73</v>
+      </c>
+      <c r="G10" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C10" t="s">
-        <v>60</v>
-      </c>
-      <c r="D10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
-        <v>6</v>
+    <row r="11" spans="1:7" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
         <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" t="s">
-        <v>72</v>
+        <v>34</v>
       </c>
       <c r="G11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
-        <v>9</v>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D12" t="s">
         <v>29</v>
       </c>
       <c r="E12" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G12" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
-        <v>5</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>55</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
         <v>29</v>
       </c>
       <c r="E13" t="s">
-        <v>38</v>
-      </c>
-      <c r="G13" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
-        <v>54</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>59</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D14" t="s">
         <v>29</v>
@@ -1672,19 +1479,16 @@
       <c r="E14" t="s">
         <v>34</v>
       </c>
-      <c r="G14" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="8" t="s">
-        <v>58</v>
+    </row>
+    <row r="15" spans="1:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>57</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
         <v>29</v>
@@ -1692,156 +1496,139 @@
       <c r="E15" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
-        <v>56</v>
+      <c r="G15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D16" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" t="s">
+        <v>37</v>
+      </c>
+      <c r="G16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C17" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" t="s">
         <v>29</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E17" t="s">
         <v>34</v>
       </c>
-      <c r="G16" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C17" t="s">
-        <v>60</v>
-      </c>
-      <c r="D17" t="s">
-        <v>36</v>
-      </c>
-      <c r="E17" t="s">
-        <v>37</v>
-      </c>
       <c r="G17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" t="s">
+        <v>62</v>
+      </c>
+      <c r="D18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" t="s">
+        <v>64</v>
+      </c>
+      <c r="G18" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C18" t="s">
-        <v>60</v>
-      </c>
-      <c r="D18" t="s">
-        <v>29</v>
-      </c>
-      <c r="E18" t="s">
-        <v>34</v>
-      </c>
-      <c r="G18" t="s">
-        <v>35</v>
-      </c>
-    </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C19" t="s">
         <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E19" t="s">
         <v>38</v>
       </c>
-      <c r="F19" t="s">
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C20" t="s">
         <v>63</v>
       </c>
-      <c r="G19" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="C20" t="s">
-        <v>60</v>
-      </c>
       <c r="D20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" t="s">
-        <v>38</v>
+        <v>20</v>
+      </c>
+      <c r="F20" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="8" t="s">
-        <v>59</v>
+      <c r="A21" s="7" t="s">
+        <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C21" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D21" t="s">
-        <v>20</v>
+        <v>67</v>
+      </c>
+      <c r="E21" t="s">
+        <v>66</v>
       </c>
       <c r="F21" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C22" t="s">
-        <v>62</v>
-      </c>
-      <c r="D22" t="s">
-        <v>66</v>
-      </c>
-      <c r="E22" t="s">
-        <v>65</v>
-      </c>
-      <c r="F22" t="s">
-        <v>73</v>
+      <c r="A22" s="8" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="8" t="s">
-        <v>23</v>
+      <c r="A23" s="7" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="8" t="s">
+      <c r="A24" s="8" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1851,257 +1638,34 @@
     <hyperlink ref="B3" r:id="rId2" xr:uid="{3504379E-CD98-4DA0-8929-22F673DFCE4A}"/>
     <hyperlink ref="B5" r:id="rId3" xr:uid="{6584CDCA-1068-4468-AF61-13CBF6BB8C9A}"/>
     <hyperlink ref="B4" r:id="rId4" xr:uid="{376368F7-01F8-4C17-AC4F-DEAF986843EA}"/>
-    <hyperlink ref="B7" r:id="rId5" xr:uid="{2650C28E-55E8-4B78-8021-073DC1D12F7D}"/>
-    <hyperlink ref="B8" r:id="rId6" xr:uid="{BBC8DDED-B21F-44E6-9B6B-88709504054F}"/>
-    <hyperlink ref="B9" r:id="rId7" xr:uid="{95A367AA-3EFF-4928-A179-84D4F2171155}"/>
-    <hyperlink ref="B13" r:id="rId8" xr:uid="{F9A7D48E-C1A7-485E-BC8B-89778E513778}"/>
-    <hyperlink ref="B14" r:id="rId9" xr:uid="{9754FBFB-0BBF-4707-9135-8E5EB4F7A374}"/>
-    <hyperlink ref="B16" r:id="rId10" xr:uid="{E8402286-6E5D-471A-BAFC-66E91A920455}"/>
-    <hyperlink ref="B11" r:id="rId11" xr:uid="{0C6AE5E9-E70A-4C03-B436-BDC499441149}"/>
-    <hyperlink ref="B17" r:id="rId12" xr:uid="{490258F2-1B04-41E0-BB78-E2D7A7A86CE0}"/>
-    <hyperlink ref="B15" r:id="rId13" xr:uid="{7FFE7EFD-C0A6-4505-9192-B1E2D7376D6B}"/>
-    <hyperlink ref="B18" r:id="rId14" xr:uid="{22C5098E-7DEF-4344-AD3C-5B19BCFBB560}"/>
-    <hyperlink ref="B21" r:id="rId15" xr:uid="{BFFF2833-9BE0-46A5-AE0D-E919A2026CBB}"/>
-    <hyperlink ref="B10" r:id="rId16" xr:uid="{4DEA275B-9985-4EB2-A90C-862012022662}"/>
-    <hyperlink ref="B12" r:id="rId17" xr:uid="{35A3109E-3672-410B-A55F-CE0E07E8B626}"/>
-    <hyperlink ref="B19" r:id="rId18" xr:uid="{5ADB7F20-9625-4010-8BDD-0EA0FE412B2B}"/>
-    <hyperlink ref="B20" r:id="rId19" xr:uid="{2DE9EE7D-9D17-4B1D-B549-98CD7CA7CD8F}"/>
-    <hyperlink ref="B22" r:id="rId20" xr:uid="{EEAFFF6C-7A6D-4625-B6D0-E5EC3672C322}"/>
-    <hyperlink ref="B6" r:id="rId21" xr:uid="{2F7F3406-1636-4D47-BD08-A874AD55D8ED}"/>
+    <hyperlink ref="B6" r:id="rId5" xr:uid="{2650C28E-55E8-4B78-8021-073DC1D12F7D}"/>
+    <hyperlink ref="B7" r:id="rId6" xr:uid="{BBC8DDED-B21F-44E6-9B6B-88709504054F}"/>
+    <hyperlink ref="B8" r:id="rId7" xr:uid="{95A367AA-3EFF-4928-A179-84D4F2171155}"/>
+    <hyperlink ref="B12" r:id="rId8" xr:uid="{F9A7D48E-C1A7-485E-BC8B-89778E513778}"/>
+    <hyperlink ref="B13" r:id="rId9" xr:uid="{9754FBFB-0BBF-4707-9135-8E5EB4F7A374}"/>
+    <hyperlink ref="B15" r:id="rId10" xr:uid="{E8402286-6E5D-471A-BAFC-66E91A920455}"/>
+    <hyperlink ref="B10" r:id="rId11" xr:uid="{0C6AE5E9-E70A-4C03-B436-BDC499441149}"/>
+    <hyperlink ref="B16" r:id="rId12" xr:uid="{490258F2-1B04-41E0-BB78-E2D7A7A86CE0}"/>
+    <hyperlink ref="B14" r:id="rId13" xr:uid="{7FFE7EFD-C0A6-4505-9192-B1E2D7376D6B}"/>
+    <hyperlink ref="B17" r:id="rId14" xr:uid="{22C5098E-7DEF-4344-AD3C-5B19BCFBB560}"/>
+    <hyperlink ref="B20" r:id="rId15" xr:uid="{BFFF2833-9BE0-46A5-AE0D-E919A2026CBB}"/>
+    <hyperlink ref="B9" r:id="rId16" xr:uid="{4DEA275B-9985-4EB2-A90C-862012022662}"/>
+    <hyperlink ref="B11" r:id="rId17" xr:uid="{35A3109E-3672-410B-A55F-CE0E07E8B626}"/>
+    <hyperlink ref="B18" r:id="rId18" xr:uid="{5ADB7F20-9625-4010-8BDD-0EA0FE412B2B}"/>
+    <hyperlink ref="B19" r:id="rId19" xr:uid="{2DE9EE7D-9D17-4B1D-B549-98CD7CA7CD8F}"/>
+    <hyperlink ref="B21" r:id="rId20" xr:uid="{EEAFFF6C-7A6D-4625-B6D0-E5EC3672C322}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId22"/>
+  <pageSetup orientation="portrait" r:id="rId21"/>
   <tableParts count="1">
-    <tablePart r:id="rId23"/>
+    <tablePart r:id="rId22"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80D50FDA-8FF9-4273-BF7A-10FE31B9AB37}">
-  <dimension ref="A1:C24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="21.21875" customWidth="1"/>
-    <col min="2" max="2" width="103.44140625" customWidth="1"/>
-    <col min="3" max="3" width="91.44140625" customWidth="1"/>
-    <col min="4" max="4" width="8.88671875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="16" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="18"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="18"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B14" s="16" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="B15" s="16" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B16" s="16" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B19" s="16" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B8" r:id="rId1" xr:uid="{0D48BC19-8A51-4CEB-9AFA-4E579070156C}"/>
-    <hyperlink ref="B9" r:id="rId2" xr:uid="{E643EBBF-95D9-4B01-AA8E-7F812464355A}"/>
-    <hyperlink ref="B10" r:id="rId3" xr:uid="{1918CB55-C36D-4A89-B948-49E256869409}"/>
-    <hyperlink ref="B13" r:id="rId4" xr:uid="{F1FE3FDC-8796-4FC5-98E0-E9EF341DBB36}"/>
-    <hyperlink ref="B14" r:id="rId5" xr:uid="{FB0B7017-402D-48E4-A27E-B33CA0AC1244}"/>
-    <hyperlink ref="B16" r:id="rId6" xr:uid="{A236F7AF-C705-41B6-B099-DFC411DA0DD0}"/>
-    <hyperlink ref="B11" r:id="rId7" xr:uid="{A57649A4-B4C9-4257-A7B1-8E15F29EEB94}"/>
-    <hyperlink ref="B12" r:id="rId8" xr:uid="{0B0A8DCD-8F15-4287-8E41-81926F924F3C}"/>
-    <hyperlink ref="B1" r:id="rId9" xr:uid="{0282B8B7-436A-4D7D-AEC1-F14BB5B630D8}"/>
-    <hyperlink ref="B15" r:id="rId10" xr:uid="{D80B71CC-4F48-498F-9AEE-BCE1E546D661}"/>
-    <hyperlink ref="B17" r:id="rId11" xr:uid="{7E599668-D83A-458E-AE50-D920729CF1EB}"/>
-    <hyperlink ref="B19" r:id="rId12" xr:uid="{A1FFC53D-552A-4EEB-9DF9-F8D1825CB868}"/>
-    <hyperlink ref="B7" r:id="rId13" xr:uid="{FD6CA973-81D6-468A-AFE1-55E842F3ECCC}"/>
-    <hyperlink ref="B2" r:id="rId14" xr:uid="{A55D131C-1979-4B34-8810-4A382A8D3787}"/>
-    <hyperlink ref="B6" r:id="rId15" xr:uid="{7B918585-13CD-4DF2-BB60-959CDA284858}"/>
-    <hyperlink ref="B5" r:id="rId16" xr:uid="{9E390795-809C-4217-A61B-8957A0FF5B09}"/>
-    <hyperlink ref="B20" r:id="rId17" xr:uid="{E403B793-807C-4569-8BA1-9872B67F7FCB}"/>
-    <hyperlink ref="B18" r:id="rId18" xr:uid="{8D45A3FB-994F-4714-9D85-A792A7C192B8}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId19"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D66BAC54-7459-4BD1-BF05-91DE6CB5AEE9}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.21875" customWidth="1"/>
@@ -2115,13 +1679,13 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D1" t="s">
         <v>24</v>
@@ -2141,10 +1705,10 @@
         <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
         <v>29</v>
@@ -2161,10 +1725,10 @@
         <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D3" t="s">
         <v>29</v>
@@ -2181,10 +1745,10 @@
         <v>12</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D4" t="s">
         <v>43</v>
@@ -2193,7 +1757,7 @@
         <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G4" t="s">
         <v>27</v>
@@ -2204,10 +1768,10 @@
         <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
         <v>29</v>
@@ -2221,136 +1785,50 @@
         <v>17</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D6" t="s">
         <v>44</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
         <v>45</v>
       </c>
-      <c r="E7" t="s">
-        <v>38</v>
+      <c r="E7" s="3" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="E8" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F9" t="s">
-        <v>30</v>
-      </c>
-      <c r="G9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D11" t="s">
-        <v>49</v>
-      </c>
-      <c r="E11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="D12" t="s">
-        <v>29</v>
-      </c>
-      <c r="E12" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -2359,141 +1837,174 @@
     <hyperlink ref="B3" r:id="rId2" xr:uid="{ADD31C52-B2C0-45BB-A957-EB0DBA57C587}"/>
     <hyperlink ref="B4" r:id="rId3" xr:uid="{8C1B4A69-7664-4743-88D5-B8B412BAB8B4}"/>
     <hyperlink ref="B5" r:id="rId4" xr:uid="{05D1AEE8-A2C3-4B67-96AD-E6F3F8372299}"/>
-    <hyperlink ref="B7" r:id="rId5" xr:uid="{3DA3698D-0749-400E-B012-09CE7EE1EE4F}"/>
-    <hyperlink ref="B8" r:id="rId6" xr:uid="{BE40119A-A51D-4D6E-A067-EA69D41567CA}"/>
-    <hyperlink ref="B9" r:id="rId7" xr:uid="{5BDC4371-380D-4C83-9763-704F260741D9}"/>
-    <hyperlink ref="B10" r:id="rId8" xr:uid="{5AB4E9A9-793B-4E63-8D97-8B217FB7E1C5}"/>
-    <hyperlink ref="B11" r:id="rId9" xr:uid="{34F6FA97-A129-456B-B5F6-BD787521ABF4}"/>
-    <hyperlink ref="B12" r:id="rId10" xr:uid="{A906FFE5-A698-4E0F-8CE1-95329052FE64}"/>
-    <hyperlink ref="B6" r:id="rId11" xr:uid="{3B4A4D12-66B2-4F76-B635-34733098B22B}"/>
+    <hyperlink ref="B6" r:id="rId5" xr:uid="{3B4A4D12-66B2-4F76-B635-34733098B22B}"/>
+    <hyperlink ref="B7" r:id="rId6" xr:uid="{709FCE77-0B89-43C8-8490-CE4B8B785DA9}"/>
+    <hyperlink ref="B8" r:id="rId7" xr:uid="{3DA3698D-0749-400E-B012-09CE7EE1EE4F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId12"/>
+  <pageSetup orientation="portrait" r:id="rId8"/>
   <tableParts count="1">
-    <tablePart r:id="rId13"/>
+    <tablePart r:id="rId9"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64225048-51D4-45F6-9E3B-46F3DE050901}">
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="90.33203125" customWidth="1"/>
+    <col min="3" max="3" width="31.33203125" customWidth="1"/>
+    <col min="4" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="43.6640625" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{D095C380-A72B-423A-B37D-7F22C532D914}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{4454D3C9-CABE-49BC-9E79-BA6DBEA6E82B}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{52046BDA-A9D1-4802-A9C9-F9834C5BD732}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{EFE8111F-E982-4785-A0FE-6FB8B133BE7B}"/>
+    <hyperlink ref="B6" r:id="rId5" xr:uid="{323E8FF9-4A14-4E02-8198-56A1CB0E59CB}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
+  <tableParts count="1">
+    <tablePart r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AE1B1A1-209E-46F9-BACB-2DF61BB6C90D}">
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="90.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="22"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="B2" s="23" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="B3" s="22" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="22"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="24" t="s">
-        <v>78</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{2270E4DC-FAB2-48FA-9DBB-EFA7C6B81913}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{DF5273A1-93C5-4938-B86A-BE96B2B2510F}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{ADC0E9AA-7299-4136-802C-0D85D208D5E6}"/>
-    <hyperlink ref="B5" r:id="rId4" xr:uid="{6B705BDA-BA26-433B-A607-4C11D01FE024}"/>
-    <hyperlink ref="B6" r:id="rId5" xr:uid="{1B32206B-536B-4FD9-B457-F1AEC0B36AA7}"/>
-    <hyperlink ref="B8" r:id="rId6" xr:uid="{83B563C5-6873-4F87-853A-B04E7097A3BB}"/>
-    <hyperlink ref="B9" r:id="rId7" xr:uid="{23BC1E69-3E17-4187-B37B-27402CFE4B30}"/>
-    <hyperlink ref="B10" r:id="rId8" xr:uid="{0E2550A4-F7A0-44A2-A9DE-896B6965C711}"/>
-    <hyperlink ref="B12" r:id="rId9" xr:uid="{A45C7993-9B95-4C15-BD88-5B57E8762A88}"/>
-    <hyperlink ref="B7" r:id="rId10" xr:uid="{83676B09-8CFC-4445-8C87-105D43677942}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE591D52-F659-41D2-A2EB-22811DA0DC42}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2505,10 +2016,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C1" t="s">
         <v>26</v>
@@ -2516,10 +2027,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
         <v>27</v>
@@ -2527,46 +2038,46 @@
     </row>
     <row r="3" spans="1:3" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" t="s">
         <v>82</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="C5" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>